<commit_message>
deploy: main → 6d188339f2b1d1789c6f047a9faa1d4a19a456ac
</commit_message>
<xml_diff>
--- a/StructureDefinition-SEEHDSLMCareDocumentationV21.xlsx
+++ b/StructureDefinition-SEEHDSLMCareDocumentationV21.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2645" uniqueCount="272">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2645" uniqueCount="274">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-10-12T12:51:47+00:00</t>
+    <t>2026-10-12T13:38:08+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -647,6 +647,10 @@
     <t>Dokument/anteckning.</t>
   </si>
   <si>
+    <t>getcaredocumentation-body-xor:Antingen clinicalDocumentNoteText eller multimediaEntry ska anges, ej båda {clinicalDocumentNoteText.exists() xor multimediaEntry.exists()}
+ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}</t>
+  </si>
+  <si>
     <t>SEEHDSLMCareDocumentationV21.careDocumentation.careDocumentationBody.clinicalDocumentNote.id</t>
   </si>
   <si>
@@ -698,6 +702,10 @@
   </si>
   <si>
     <t>Dokumentets innehåll i form av en multimediaobjekt, i form av antingen ett inbäddat objekt eller en länk till objektet. Obs Man kan välja att skicka dokumentets innehåll i elementet clinicalDocumentNoteText eller i multimediaEntry enligt respektive elements regler, man får inte skicka med båda elementen. Regeln finns med i constraints.xml(schematron) under katalogen test-suites och kan valideras med testsviten.</t>
+  </si>
+  <si>
+    <t>getcaredocumentation-multimedia-xor:Antingen value eller reference ska anges i multimediaEntry, ej båda {value.exists() xor reference.exists()}
+ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}</t>
   </si>
   <si>
     <t>SEEHDSLMCareDocumentationV21.careDocumentation.careDocumentationBody.clinicalDocumentNote.multimediaEntry.id</t>
@@ -6339,15 +6347,15 @@
         <v>72</v>
       </c>
       <c r="AJ51" t="s" s="2">
-        <v>81</v>
+        <v>204</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s" s="2">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
@@ -6444,10 +6452,10 @@
     </row>
     <row r="53">
       <c r="A53" t="s" s="2">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
@@ -6546,10 +6554,10 @@
     </row>
     <row r="54">
       <c r="A54" t="s" s="2">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" t="s" s="2">
@@ -6650,10 +6658,10 @@
     </row>
     <row r="55">
       <c r="A55" t="s" s="2">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
@@ -6679,10 +6687,10 @@
         <v>112</v>
       </c>
       <c r="L55" t="s" s="2">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="M55" t="s" s="2">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="N55" s="2"/>
       <c r="O55" s="2"/>
@@ -6733,7 +6741,7 @@
         <v>72</v>
       </c>
       <c r="AF55" t="s" s="2">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AG55" t="s" s="2">
         <v>73</v>
@@ -6750,10 +6758,10 @@
     </row>
     <row r="56">
       <c r="A56" t="s" s="2">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" t="s" s="2">
@@ -6779,10 +6787,10 @@
         <v>112</v>
       </c>
       <c r="L56" t="s" s="2">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="M56" t="s" s="2">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="N56" s="2"/>
       <c r="O56" s="2"/>
@@ -6833,7 +6841,7 @@
         <v>72</v>
       </c>
       <c r="AF56" t="s" s="2">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="AG56" t="s" s="2">
         <v>73</v>
@@ -6850,10 +6858,10 @@
     </row>
     <row r="57">
       <c r="A57" t="s" s="2">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" t="s" s="2">
@@ -6879,10 +6887,10 @@
         <v>112</v>
       </c>
       <c r="L57" t="s" s="2">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="M57" t="s" s="2">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="N57" s="2"/>
       <c r="O57" s="2"/>
@@ -6933,7 +6941,7 @@
         <v>72</v>
       </c>
       <c r="AF57" t="s" s="2">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AG57" t="s" s="2">
         <v>73</v>
@@ -6950,10 +6958,10 @@
     </row>
     <row r="58">
       <c r="A58" t="s" s="2">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" t="s" s="2">
@@ -6979,10 +6987,10 @@
         <v>112</v>
       </c>
       <c r="L58" t="s" s="2">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="M58" t="s" s="2">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="N58" s="2"/>
       <c r="O58" s="2"/>
@@ -7033,7 +7041,7 @@
         <v>72</v>
       </c>
       <c r="AF58" t="s" s="2">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="AG58" t="s" s="2">
         <v>73</v>
@@ -7050,10 +7058,10 @@
     </row>
     <row r="59">
       <c r="A59" t="s" s="2">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" t="s" s="2">
@@ -7079,10 +7087,10 @@
         <v>78</v>
       </c>
       <c r="L59" t="s" s="2">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="M59" t="s" s="2">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="N59" s="2"/>
       <c r="O59" s="2"/>
@@ -7133,7 +7141,7 @@
         <v>72</v>
       </c>
       <c r="AF59" t="s" s="2">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="AG59" t="s" s="2">
         <v>73</v>
@@ -7145,15 +7153,15 @@
         <v>72</v>
       </c>
       <c r="AJ59" t="s" s="2">
-        <v>81</v>
+        <v>222</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="s" s="2">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C60" s="2"/>
       <c r="D60" t="s" s="2">
@@ -7250,10 +7258,10 @@
     </row>
     <row r="61">
       <c r="A61" t="s" s="2">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" t="s" s="2">
@@ -7352,10 +7360,10 @@
     </row>
     <row r="62">
       <c r="A62" t="s" s="2">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B62" t="s" s="2">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="C62" s="2"/>
       <c r="D62" t="s" s="2">
@@ -7456,10 +7464,10 @@
     </row>
     <row r="63">
       <c r="A63" t="s" s="2">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B63" t="s" s="2">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C63" s="2"/>
       <c r="D63" t="s" s="2">
@@ -7485,10 +7493,10 @@
         <v>112</v>
       </c>
       <c r="L63" t="s" s="2">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="M63" t="s" s="2">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="N63" s="2"/>
       <c r="O63" s="2"/>
@@ -7539,7 +7547,7 @@
         <v>72</v>
       </c>
       <c r="AF63" t="s" s="2">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="AG63" t="s" s="2">
         <v>83</v>
@@ -7556,10 +7564,10 @@
     </row>
     <row r="64">
       <c r="A64" t="s" s="2">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B64" t="s" s="2">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C64" s="2"/>
       <c r="D64" t="s" s="2">
@@ -7582,13 +7590,13 @@
         <v>72</v>
       </c>
       <c r="K64" t="s" s="2">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="L64" t="s" s="2">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="M64" t="s" s="2">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="N64" s="2"/>
       <c r="O64" s="2"/>
@@ -7639,7 +7647,7 @@
         <v>72</v>
       </c>
       <c r="AF64" t="s" s="2">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="AG64" t="s" s="2">
         <v>73</v>
@@ -7656,10 +7664,10 @@
     </row>
     <row r="65">
       <c r="A65" t="s" s="2">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B65" t="s" s="2">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C65" s="2"/>
       <c r="D65" t="s" s="2">
@@ -7682,13 +7690,13 @@
         <v>72</v>
       </c>
       <c r="K65" t="s" s="2">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="L65" t="s" s="2">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="M65" t="s" s="2">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="N65" s="2"/>
       <c r="O65" s="2"/>
@@ -7739,7 +7747,7 @@
         <v>72</v>
       </c>
       <c r="AF65" t="s" s="2">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="AG65" t="s" s="2">
         <v>73</v>
@@ -7756,10 +7764,10 @@
     </row>
     <row r="66">
       <c r="A66" t="s" s="2">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B66" t="s" s="2">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="C66" s="2"/>
       <c r="D66" t="s" s="2">
@@ -7785,10 +7793,10 @@
         <v>78</v>
       </c>
       <c r="L66" t="s" s="2">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="M66" t="s" s="2">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="N66" s="2"/>
       <c r="O66" s="2"/>
@@ -7839,7 +7847,7 @@
         <v>72</v>
       </c>
       <c r="AF66" t="s" s="2">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="AG66" t="s" s="2">
         <v>73</v>
@@ -7856,10 +7864,10 @@
     </row>
     <row r="67">
       <c r="A67" t="s" s="2">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B67" t="s" s="2">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C67" s="2"/>
       <c r="D67" t="s" s="2">
@@ -7956,10 +7964,10 @@
     </row>
     <row r="68">
       <c r="A68" t="s" s="2">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B68" t="s" s="2">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="C68" s="2"/>
       <c r="D68" t="s" s="2">
@@ -8058,10 +8066,10 @@
     </row>
     <row r="69">
       <c r="A69" t="s" s="2">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B69" t="s" s="2">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="C69" s="2"/>
       <c r="D69" t="s" s="2">
@@ -8162,10 +8170,10 @@
     </row>
     <row r="70">
       <c r="A70" t="s" s="2">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B70" t="s" s="2">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="C70" s="2"/>
       <c r="D70" t="s" s="2">
@@ -8188,13 +8196,13 @@
         <v>72</v>
       </c>
       <c r="K70" t="s" s="2">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="L70" t="s" s="2">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="M70" t="s" s="2">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="N70" s="2"/>
       <c r="O70" s="2"/>
@@ -8245,7 +8253,7 @@
         <v>72</v>
       </c>
       <c r="AF70" t="s" s="2">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="AG70" t="s" s="2">
         <v>73</v>
@@ -8262,10 +8270,10 @@
     </row>
     <row r="71">
       <c r="A71" t="s" s="2">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B71" t="s" s="2">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="C71" s="2"/>
       <c r="D71" t="s" s="2">
@@ -8291,7 +8299,7 @@
         <v>122</v>
       </c>
       <c r="L71" t="s" s="2">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="M71" t="s" s="2">
         <v>180</v>
@@ -8345,7 +8353,7 @@
         <v>72</v>
       </c>
       <c r="AF71" t="s" s="2">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="AG71" t="s" s="2">
         <v>83</v>
@@ -8362,10 +8370,10 @@
     </row>
     <row r="72">
       <c r="A72" t="s" s="2">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B72" t="s" s="2">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="C72" s="2"/>
       <c r="D72" t="s" s="2">
@@ -8391,10 +8399,10 @@
         <v>112</v>
       </c>
       <c r="L72" t="s" s="2">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="M72" t="s" s="2">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="N72" s="2"/>
       <c r="O72" s="2"/>
@@ -8445,7 +8453,7 @@
         <v>72</v>
       </c>
       <c r="AF72" t="s" s="2">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="AG72" t="s" s="2">
         <v>83</v>
@@ -8462,10 +8470,10 @@
     </row>
     <row r="73">
       <c r="A73" t="s" s="2">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B73" t="s" s="2">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="C73" s="2"/>
       <c r="D73" t="s" s="2">
@@ -8491,10 +8499,10 @@
         <v>126</v>
       </c>
       <c r="L73" t="s" s="2">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="M73" t="s" s="2">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="N73" s="2"/>
       <c r="O73" s="2"/>
@@ -8545,7 +8553,7 @@
         <v>72</v>
       </c>
       <c r="AF73" t="s" s="2">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="AG73" t="s" s="2">
         <v>83</v>
@@ -8562,10 +8570,10 @@
     </row>
     <row r="74">
       <c r="A74" t="s" s="2">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B74" t="s" s="2">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="C74" s="2"/>
       <c r="D74" t="s" s="2">
@@ -8591,10 +8599,10 @@
         <v>112</v>
       </c>
       <c r="L74" t="s" s="2">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="M74" t="s" s="2">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="N74" s="2"/>
       <c r="O74" s="2"/>
@@ -8645,7 +8653,7 @@
         <v>72</v>
       </c>
       <c r="AF74" t="s" s="2">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="AG74" t="s" s="2">
         <v>83</v>
@@ -8662,10 +8670,10 @@
     </row>
     <row r="75">
       <c r="A75" t="s" s="2">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B75" t="s" s="2">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="C75" s="2"/>
       <c r="D75" t="s" s="2">
@@ -8691,10 +8699,10 @@
         <v>78</v>
       </c>
       <c r="L75" t="s" s="2">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="M75" t="s" s="2">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="N75" s="2"/>
       <c r="O75" s="2"/>
@@ -8745,7 +8753,7 @@
         <v>72</v>
       </c>
       <c r="AF75" t="s" s="2">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AG75" t="s" s="2">
         <v>83</v>
@@ -8762,10 +8770,10 @@
     </row>
     <row r="76">
       <c r="A76" t="s" s="2">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B76" t="s" s="2">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="C76" s="2"/>
       <c r="D76" t="s" s="2">
@@ -8862,10 +8870,10 @@
     </row>
     <row r="77">
       <c r="A77" t="s" s="2">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B77" t="s" s="2">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="C77" s="2"/>
       <c r="D77" t="s" s="2">
@@ -8964,10 +8972,10 @@
     </row>
     <row r="78">
       <c r="A78" t="s" s="2">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B78" t="s" s="2">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="C78" s="2"/>
       <c r="D78" t="s" s="2">
@@ -9068,10 +9076,10 @@
     </row>
     <row r="79">
       <c r="A79" t="s" s="2">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B79" t="s" s="2">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="C79" s="2"/>
       <c r="D79" t="s" s="2">
@@ -9097,10 +9105,10 @@
         <v>112</v>
       </c>
       <c r="L79" t="s" s="2">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="M79" t="s" s="2">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="N79" s="2"/>
       <c r="O79" s="2"/>
@@ -9151,7 +9159,7 @@
         <v>72</v>
       </c>
       <c r="AF79" t="s" s="2">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="AG79" t="s" s="2">
         <v>83</v>
@@ -9168,10 +9176,10 @@
     </row>
     <row r="80">
       <c r="A80" t="s" s="2">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B80" t="s" s="2">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="C80" s="2"/>
       <c r="D80" t="s" s="2">
@@ -9197,10 +9205,10 @@
         <v>112</v>
       </c>
       <c r="L80" t="s" s="2">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="M80" t="s" s="2">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="N80" s="2"/>
       <c r="O80" s="2"/>
@@ -9251,7 +9259,7 @@
         <v>72</v>
       </c>
       <c r="AF80" t="s" s="2">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="AG80" t="s" s="2">
         <v>73</v>
@@ -9268,10 +9276,10 @@
     </row>
     <row r="81">
       <c r="A81" t="s" s="2">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B81" t="s" s="2">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="C81" s="2"/>
       <c r="D81" t="s" s="2">
@@ -9297,10 +9305,10 @@
         <v>112</v>
       </c>
       <c r="L81" t="s" s="2">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="M81" t="s" s="2">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="N81" s="2"/>
       <c r="O81" s="2"/>
@@ -9351,7 +9359,7 @@
         <v>72</v>
       </c>
       <c r="AF81" t="s" s="2">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="AG81" t="s" s="2">
         <v>83</v>
@@ -9368,10 +9376,10 @@
     </row>
     <row r="82">
       <c r="A82" t="s" s="2">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B82" t="s" s="2">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C82" s="2"/>
       <c r="D82" t="s" s="2">
@@ -9397,10 +9405,10 @@
         <v>112</v>
       </c>
       <c r="L82" t="s" s="2">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="M82" t="s" s="2">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="N82" s="2"/>
       <c r="O82" s="2"/>
@@ -9451,7 +9459,7 @@
         <v>72</v>
       </c>
       <c r="AF82" t="s" s="2">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="AG82" t="s" s="2">
         <v>73</v>
@@ -9468,10 +9476,10 @@
     </row>
     <row r="83">
       <c r="A83" t="s" s="2">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B83" t="s" s="2">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="C83" s="2"/>
       <c r="D83" t="s" s="2">
@@ -9497,10 +9505,10 @@
         <v>112</v>
       </c>
       <c r="L83" t="s" s="2">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="M83" t="s" s="2">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="N83" s="2"/>
       <c r="O83" s="2"/>
@@ -9551,7 +9559,7 @@
         <v>72</v>
       </c>
       <c r="AF83" t="s" s="2">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="AG83" t="s" s="2">
         <v>73</v>

</xml_diff>